<commit_message>
feat(testing): display unassigned Sprint values
Source: artifacts/unassigned-sprint-display-plan-20261014.html
</commit_message>
<xml_diff>
--- a/docs/testing/PROJECT TEST CASES CAA 141026.xlsx
+++ b/docs/testing/PROJECT TEST CASES CAA 141026.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="TEST CASES" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TEST CASES" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
   <dimension ref="A1:J355"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="32" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
@@ -3148,7 +3148,11 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="inlineStr"/>
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
           <t>E02-S05</t>
@@ -3198,7 +3202,11 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="inlineStr"/>
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
           <t>E02-S05</t>
@@ -3247,7 +3255,11 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="2" t="inlineStr"/>
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
           <t>E02-S05</t>
@@ -3297,7 +3309,11 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="2" t="inlineStr"/>
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
           <t>E02-S07</t>
@@ -3346,7 +3362,11 @@
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="2" t="inlineStr"/>
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
           <t>E02-S07</t>
@@ -3395,7 +3415,11 @@
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="2" t="inlineStr"/>
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
           <t>E02-S07</t>
@@ -3444,7 +3468,11 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="inlineStr"/>
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
           <t>E02-S07</t>
@@ -3493,7 +3521,11 @@
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="2" t="inlineStr"/>
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
           <t>E02-S07</t>
@@ -6274,7 +6306,11 @@
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="2" t="inlineStr"/>
+      <c r="A113" s="2" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
           <t>E04-S02</t>
@@ -6323,7 +6359,11 @@
       </c>
     </row>
     <row r="114">
-      <c r="A114" s="2" t="inlineStr"/>
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
           <t>E04-S02</t>
@@ -6373,7 +6413,11 @@
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="2" t="inlineStr"/>
+      <c r="A115" s="2" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
           <t>E04-S02</t>
@@ -6423,7 +6467,11 @@
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="2" t="inlineStr"/>
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
           <t>E04-S02</t>
@@ -6473,7 +6521,11 @@
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="2" t="inlineStr"/>
+      <c r="A117" s="2" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
           <t>E04-S02</t>
@@ -12070,7 +12122,11 @@
       </c>
     </row>
     <row r="223">
-      <c r="A223" s="2" t="inlineStr"/>
+      <c r="A223" s="2" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
       <c r="B223" s="2" t="inlineStr">
         <is>
           <t>E07-S08</t>
@@ -12120,7 +12176,11 @@
       </c>
     </row>
     <row r="224">
-      <c r="A224" s="2" t="inlineStr"/>
+      <c r="A224" s="2" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
       <c r="B224" s="2" t="inlineStr">
         <is>
           <t>E07-S08</t>
@@ -12169,7 +12229,11 @@
       </c>
     </row>
     <row r="225">
-      <c r="A225" s="2" t="inlineStr"/>
+      <c r="A225" s="2" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
       <c r="B225" s="2" t="inlineStr">
         <is>
           <t>E07-S08</t>
@@ -12218,7 +12282,11 @@
       </c>
     </row>
     <row r="226">
-      <c r="A226" s="2" t="inlineStr"/>
+      <c r="A226" s="2" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
       <c r="B226" s="2" t="inlineStr">
         <is>
           <t>E07-S08</t>
@@ -16955,7 +17023,11 @@
       </c>
     </row>
     <row r="317">
-      <c r="A317" s="2" t="inlineStr"/>
+      <c r="A317" s="2" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
       <c r="B317" s="2" t="inlineStr">
         <is>
           <t>E10-S03</t>
@@ -17004,7 +17076,11 @@
       </c>
     </row>
     <row r="318">
-      <c r="A318" s="2" t="inlineStr"/>
+      <c r="A318" s="2" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
       <c r="B318" s="2" t="inlineStr">
         <is>
           <t>E10-S03</t>
@@ -17053,7 +17129,11 @@
       </c>
     </row>
     <row r="319">
-      <c r="A319" s="2" t="inlineStr"/>
+      <c r="A319" s="2" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
       <c r="B319" s="2" t="inlineStr">
         <is>
           <t>E10-S03</t>
@@ -17102,7 +17182,11 @@
       </c>
     </row>
     <row r="320">
-      <c r="A320" s="2" t="inlineStr"/>
+      <c r="A320" s="2" t="inlineStr">
+        <is>
+          <t>Unassigned</t>
+        </is>
+      </c>
       <c r="B320" s="2" t="inlineStr">
         <is>
           <t>E10-S03</t>

</xml_diff>

<commit_message>
docs(testing): regenerate seeded fixture exports
</commit_message>
<xml_diff>
--- a/docs/testing/PROJECT TEST CASES CAA 141026.xlsx
+++ b/docs/testing/PROJECT TEST CASES CAA 141026.xlsx
@@ -6713,7 +6713,7 @@
       </c>
       <c r="G121" s="2" t="inlineStr">
         <is>
-          <t>Orchid Hall has the seeded future Pending booking for "EVT-3003 Planning Phase Gala" on 25/10/2026 18:00-22:00</t>
+          <t>Orchid Hall has the seeded booking for "EVT-3003 Planning Phase Gala" on 25/10/2026 18:00-22:00. For this case only, prepare that future booking as Confirmed before attempting retirement</t>
         </is>
       </c>
       <c r="H121" s="2" t="inlineStr">
@@ -6725,12 +6725,12 @@
       </c>
       <c r="I121" s="2" t="inlineStr">
         <is>
-          <t>Venue: Orchid Hall | Blocking booking: EVT-3003 Planning Phase Gala, Pending, 25/10/2026 18:00-22:00</t>
+          <t>Venue: Orchid Hall | Blocking booking: EVT-3003 Planning Phase Gala, Confirmed, 25/10/2026 18:00-22:00</t>
         </is>
       </c>
       <c r="J121" s="2" t="inlineStr">
         <is>
-          <t>Retirement is blocked with a message identifying the Pending booking for "EVT-3003 Planning Phase Gala" on 25/10/2026 as the reason</t>
+          <t>Retirement is blocked with a message identifying the Confirmed booking for "EVT-3003 Planning Phase Gala" on 25/10/2026 as the reason</t>
         </is>
       </c>
     </row>
@@ -9453,27 +9453,27 @@
       </c>
       <c r="G173" s="2" t="inlineStr">
         <is>
-          <t>"EVT-3003 Planning Phase Gala" is the seeded Planning event assigned to coord_a@connectsphere.com; its seeded Orchid Hall booking is Pending on 25/10/2026 18:00-22:00 and is linked to its compatibility Session. Cedar Auditorium is free and its Banquet capacity 250 exceeds the event's expected attendance 200</t>
+          <t>"EVT-3003 Planning Phase Gala" is the seeded Planning event assigned to coord_a@connectsphere.com with expected attendance 200 and a compatibility Session on 25/10/2026 18:00-22:00. For this case only, prepare its Pending request at Lotus Room, whose maximum capacity 50 and Boardroom capacity 40 are below 200. Cedar Auditorium is free and its Banquet capacity 250 exceeds 200</t>
         </is>
       </c>
       <c r="H173" s="2" t="inlineStr">
         <is>
           <t>1. Log in as venue_a@connectsphere.com
-  2. Open the Pending request for "EVT-3003 Planning Phase Gala" at Orchid Hall
+  2. Open the Pending request for "EVT-3003 Planning Phase Gala" at Lotus Room
   3. Click "Reject"
-  4. Enter reason "Venue cannot meet the event's requirements" and suggest alternative venue "Cedar Auditorium"
+  4. Enter reason "Capacity too small for expected attendance" and suggest alternative venue "Cedar Auditorium"
   5. Confirm the rejection
   6. Log in as the assigned Coordinator and check the notification and request</t>
         </is>
       </c>
       <c r="I173" s="2" t="inlineStr">
         <is>
-          <t>Event: EVT-3003 Planning Phase Gala | Rejection reason: "Venue cannot meet the event's requirements" | Suggested alternative: Cedar Auditorium</t>
+          <t>Event: EVT-3003 Planning Phase Gala | Requested venue: Lotus Room (maximum 50; Boardroom 40) | Expected attendance: 200 | Rejection reason: "Capacity too small for expected attendance" | Suggested alternative: Cedar Auditorium (Banquet 250)</t>
         </is>
       </c>
       <c r="J173" s="2" t="inlineStr">
         <is>
-          <t>coord_a@connectsphere.com is notified with the rejection reason and suggested Cedar Auditorium alternative. The rejected booking remains recorded, and the Coordinator can submit a replacement request using the suggestion without restarting the venue search</t>
+          <t>coord_a@connectsphere.com is notified with the exact capacity reason and suggested Cedar Auditorium alternative. The rejected Lotus Room booking remains recorded, and the Coordinator can amend the existing request to Cedar Auditorium without restarting the venue search</t>
         </is>
       </c>
     </row>

</xml_diff>